<commit_message>
Add identity cards for officers selected in the 2nd randomisation
- New Identity Cards page in the left menu (Output): party-wise and
  duty-wise cards, 8 per A4 page, PDF via print
- Cards only for officers in locked 2nd-randomisation parts
- QR code (embedded qrcode-generator, MIT), signature from Setup,
  editable heading and signatory label
- Optional Blood Group officer column (Excel import/export, templates)
- Fixed-size cards with shrink-to-fit text; e2e tests decode every QR
  with jsQR and check counts, order, gating and page count

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5zeq2JHM1LeQHsBokCXrg
</commit_message>
<xml_diff>
--- a/test-data/Officers_Template.xlsx
+++ b/test-data/Officers_Template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:Q4"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -416,6 +416,7 @@
     <col min="14" max="14" width="14.83203125" customWidth="1"/>
     <col min="15" max="15" width="14.83203125" customWidth="1"/>
     <col min="16" max="16" width="13.83203125" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,6 +468,9 @@
       <c r="P1" t="str">
         <v>IFSC</v>
       </c>
+      <c r="Q1" t="str">
+        <v>Blood Group</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -517,6 +521,9 @@
       <c r="P2" t="str">
         <v>SBIN0000001</v>
       </c>
+      <c r="Q2" t="str">
+        <v>B+</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -620,14 +627,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -707,9 +714,14 @@
         <v>Account No, Bank, Branch, IFSC — optional; printed on training attendance sheets.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Blood Group — optional; printed on the identity card when filled.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>